<commit_message>
Update data package at: 2026-09-25T12:14:42Z
</commit_message>
<xml_diff>
--- a/data-raw/desc_Setor_UO_Orgao.xlsx
+++ b/data-raw/desc_Setor_UO_Orgao.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\x1569275\CAMG\Splor Geral - @dcppn\00- DCPPN 2027\PPAG e LOA 2027\Dados para Volumes\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_67BEBA03C2A83042867FE281EC8FE06AF5979440" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Setor_UO_Órgão" sheetId="1" r:id="rId1"/>
@@ -17,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Setor_UO_Órgão!$A$1:$E$122</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -61,6 +62,9 @@
     <t>ADVOCACIA GERAL</t>
   </si>
   <si>
+    <t>FUNDO ESPECIAL DA ADVOCACIA-GERAL DO ESTADO</t>
+  </si>
+  <si>
     <t>SECRETARIA DE ESTADO DE AGRICULTURA, PECUÁRIA E ABASTECIMENTO</t>
   </si>
   <si>
@@ -88,6 +92,9 @@
     <t>INSTITUTO DE PREVIDÊNCIA DO LEGISLATIVO DO ESTADO DE MINAS GERAIS</t>
   </si>
   <si>
+    <t>FUNDO ESPECIAL DA ASSEMBLEIA LEGISLATIVA DO ESTADO DE MINAS GERAIS</t>
+  </si>
+  <si>
     <t>SECRETARIA DE ESTADO DA CASA CIVIL</t>
   </si>
   <si>
@@ -145,6 +152,9 @@
     <t>DEFENSORIA PÚBLICA</t>
   </si>
   <si>
+    <t xml:space="preserve">FUNDO ESPECIAL DE GARANTIA DE ACESSO À JUSTIÇA </t>
+  </si>
+  <si>
     <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO</t>
   </si>
   <si>
@@ -313,6 +323,39 @@
     <t>GOVERNO</t>
   </si>
   <si>
+    <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIAS</t>
+  </si>
+  <si>
+    <t>INFRAESTRUTURA, MOBILIDADE E PARCERIAS</t>
+  </si>
+  <si>
+    <t>DEPARTAMENTO DE ESTRADAS DE RODAGEM DO ESTADO DE MINAS GERAIS</t>
+  </si>
+  <si>
+    <t>AGÊNCIA DE DESENVOLVIMENTO DA REGIÃO METROPOLITANA DE BELO HORIZONTE</t>
+  </si>
+  <si>
+    <t>AGÊNCIA DE DESENVOLVIMENTO DA REGIÃO METROPOLITANA DO VALE DO AÇO</t>
+  </si>
+  <si>
+    <t>FUNDO DE DESENVOLVIMENTO METROPOLITANO</t>
+  </si>
+  <si>
+    <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
+  </si>
+  <si>
+    <t>FUNDO DE PAGAMENTO DE PARCERIAS PÚBLICO - PRIVADAS DE MINAS GERAIS</t>
+  </si>
+  <si>
+    <t>FUNDO DE GARANTIAS DE PARCERIAS PÚBLICO - PRIVADAS DE MINAS GERAIS</t>
+  </si>
+  <si>
+    <t>TREM METROPOLITANO DE BELO HORIZONTE S.A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGÊNCIA REGULADORA DE TRANSPORTES DO ESTADO DE MINAS GERAIS </t>
+  </si>
+  <si>
     <t>SECRETARIA DE ESTADO DE JUSTIÇA E SEGURANÇA PÚBLICA</t>
   </si>
   <si>
@@ -349,18 +392,27 @@
     <t>FUNDO DE RECUPERAÇÃO, PROTEÇÃO E DESENVOLVIMENTO SUSTENTÁVEL DAS BACIAS HIDROGRÁFICAS DO ESTADO DE MINAS GERAIS</t>
   </si>
   <si>
+    <t>FUNDO ESTADUAL DE SANEAMENTO BÁSICO DE MINAS GERAIS</t>
+  </si>
+  <si>
     <t>PROCURADORIA GERAL DE JUSTIÇA</t>
   </si>
   <si>
     <t>MINISTÉRIO PÚBLICO</t>
   </si>
   <si>
+    <t>MINISTÉRIO PÚBLICO DO ESTADO DE MINAS GERAIS</t>
+  </si>
+  <si>
     <t>FUNDO ESPECIAL DO MINISTÉRIO PÚBLICO DO ESTADO DE MINAS GERAIS</t>
   </si>
   <si>
     <t>FUNDO ESTADUAL DE PROTEÇÃO E DEFESA DO CONSUMIDOR</t>
   </si>
   <si>
+    <t>FUNDO DE DESENVOLVIMENTO DO MINISTÉRIO PÚBLICO</t>
+  </si>
+  <si>
     <t>OUVIDORIA-GERAL DO ESTADO DE MINAS GERAIS</t>
   </si>
   <si>
@@ -394,6 +446,9 @@
     <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS</t>
   </si>
   <si>
+    <t>DEPARTAMENTO ESTADUAL DE TRÂNSITO DE MINAS GERAIS</t>
+  </si>
+  <si>
     <t>POLÍCIA CIVIL DO ESTADO DE MINAS GERAIS</t>
   </si>
   <si>
@@ -427,33 +482,6 @@
     <t>FUNDO ESTADUAL DE SAÚDE</t>
   </si>
   <si>
-    <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIAS</t>
-  </si>
-  <si>
-    <t>INFRAESTRUTURA, MOBILIDADE E PARCERIAS</t>
-  </si>
-  <si>
-    <t>AGÊNCIA DE DESENVOLVIMENTO DA REGIÃO METROPOLITANA DE BELO HORIZONTE</t>
-  </si>
-  <si>
-    <t>AGÊNCIA DE DESENVOLVIMENTO DA REGIÃO METROPOLITANA DO VALE DO AÇO</t>
-  </si>
-  <si>
-    <t>FUNDO DE DESENVOLVIMENTO METROPOLITANO</t>
-  </si>
-  <si>
-    <t>FUNDO ESTADUAL DE DESENVOLVIMENTO DE TRANSPORTES</t>
-  </si>
-  <si>
-    <t>FUNDO DE PAGAMENTO DE PARCERIAS PÚBLICO - PRIVADAS DE MINAS GERAIS</t>
-  </si>
-  <si>
-    <t>FUNDO DE GARANTIAS DE PARCERIAS PÚBLICO - PRIVADAS DE MINAS GERAIS</t>
-  </si>
-  <si>
-    <t>TREM METROPOLITANO DE BELO HORIZONTE S.A</t>
-  </si>
-  <si>
     <t>TRIBUNAL DE CONTAS DO ESTADO DE MINAS GERAIS</t>
   </si>
   <si>
@@ -476,40 +504,13 @@
   </si>
   <si>
     <t>TRIBUNAL DE JUSTIÇA MILITAR</t>
-  </si>
-  <si>
-    <t>FUNDO DE DESENVOLVIMENTO DO MINISTÉRIO PÚBLICO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FUNDO ESPECIAL DE GARANTIA DE ACESSO À JUSTIÇA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AGÊNCIA REGULADORA DE TRANSPORTES DO ESTADO DE MINAS GERAIS </t>
-  </si>
-  <si>
-    <t>FUNDO ESPECIAL DA ASSEMBLEIA LEGISLATIVA DO ESTADO DE MINAS GERAIS</t>
-  </si>
-  <si>
-    <t>DEPARTAMENTO DE ESTRADAS DE RODAGEM DO ESTADO DE MINAS GERAIS</t>
-  </si>
-  <si>
-    <t>DEPARTAMENTO ESTADUAL DE TRÂNSITO DE MINAS GERAIS</t>
-  </si>
-  <si>
-    <t>FUNDO ESTADUAL DE SANEAMENTO BÁSICO DE MINAS GERAIS</t>
-  </si>
-  <si>
-    <t>MINISTÉRIO PÚBLICO DO ESTADO DE MINAS GERAIS</t>
-  </si>
-  <si>
-    <t>FUNDO ESPECIAL DA ADVOCACIA-GERAL DO ESTADO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -610,16 +611,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:E122" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <sortState ref="A2:E122">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabela2" displayName="Tabela2" ref="A1:E122" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E122">
     <sortCondition ref="C1:C122"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="1" name="Cód. UO Ação" dataDxfId="4"/>
-    <tableColumn id="2" name="UO Ação" dataDxfId="3"/>
-    <tableColumn id="3" name="Setor de Governo" dataDxfId="2"/>
-    <tableColumn id="4" name="Cód Órgão" dataDxfId="1"/>
-    <tableColumn id="5" name="Descrição Órgão" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Cód. UO Ação" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="UO Ação" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Setor de Governo" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Cód Órgão" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Descrição Órgão" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -921,9 +922,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E122"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="63" style="1" customWidth="1"/>
@@ -932,7 +933,7 @@
     <col min="5" max="5" width="73.42578125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -949,7 +950,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5">
       <c r="A2" s="1">
         <v>1081</v>
       </c>
@@ -966,12 +967,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5">
       <c r="A3" s="1">
         <v>4751</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>154</v>
+        <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -983,2027 +984,2027 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5">
       <c r="A4" s="1">
         <v>1231</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D4" s="1">
         <v>1230</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" s="1">
         <v>2371</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="D5" s="1">
         <v>1230</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" s="1">
         <v>3041</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D6" s="1">
         <v>1230</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" s="1">
         <v>3051</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D7" s="1">
         <v>1230</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" s="1">
         <v>4171</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D8" s="1">
         <v>1230</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9" s="1">
         <v>1011</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D9" s="1">
         <v>1010</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10" s="1">
         <v>2361</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="D10" s="1">
         <v>1010</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11" s="1">
         <v>4121</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>149</v>
+        <v>17</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D11" s="1">
         <v>1010</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
       <c r="A12" s="1">
         <v>1721</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D12" s="1">
         <v>1720</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
       <c r="A13" s="1">
         <v>1951</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D13" s="1">
         <v>1720</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
       <c r="A14" s="1">
         <v>1711</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D14" s="1">
         <v>1710</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
       <c r="A15" s="1">
         <v>2211</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D15" s="1">
         <v>1710</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
       <c r="A16" s="1">
         <v>3151</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="D16" s="1">
         <v>1710</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
       <c r="A17" s="1">
         <v>1521</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D17" s="1">
         <v>1520</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
       <c r="A18" s="1">
         <v>1401</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D18" s="1">
         <v>1400</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
       <c r="A19" s="1">
         <v>1271</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D19" s="1">
         <v>1270</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
       <c r="A20" s="1">
         <v>2171</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D20" s="1">
         <v>1270</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
       <c r="A21" s="1">
         <v>2181</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="D21" s="1">
         <v>1270</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
       <c r="A22" s="1">
         <v>2201</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D22" s="1">
         <v>1270</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
       <c r="A23" s="1">
         <v>4151</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D23" s="1">
         <v>1270</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
       <c r="A24" s="1">
         <v>4491</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D24" s="1">
         <v>1270</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
       <c r="A25" s="1">
         <v>1441</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D25" s="1">
         <v>1440</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
       <c r="A26" s="1">
         <v>4741</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>147</v>
+        <v>37</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D26" s="1">
         <v>1440</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
       <c r="A27" s="1">
         <v>1221</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D27" s="1">
         <v>1220</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
       <c r="A28" s="1">
         <v>2041</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D28" s="1">
         <v>1220</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
       <c r="A29" s="1">
         <v>2071</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D29" s="1">
         <v>1220</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
       <c r="A30" s="1">
         <v>2251</v>
       </c>
       <c r="B30" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="D30" s="1">
         <v>1220</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
       <c r="A31" s="1">
         <v>4111</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D31" s="1">
         <v>1220</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
       <c r="A32" s="1">
         <v>4531</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D32" s="1">
         <v>1220</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
       <c r="A33" s="1">
         <v>4661</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D33" s="1">
         <v>1220</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
       <c r="A34" s="1">
         <v>4671</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D34" s="1">
         <v>1220</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
       <c r="A35" s="1">
         <v>5011</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D35" s="1">
         <v>1220</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
       <c r="A36" s="1">
         <v>5031</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D36" s="1">
         <v>1220</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
       <c r="A37" s="1">
         <v>5071</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D37" s="1">
         <v>1220</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
       <c r="A38" s="1">
         <v>5081</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D38" s="1">
         <v>1220</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
       <c r="A39" s="1">
         <v>5121</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D39" s="1">
         <v>1220</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
       <c r="A40" s="2">
         <v>5131</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D40" s="2">
         <v>1220</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
       <c r="A41" s="1">
         <v>5191</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D41" s="1">
         <v>1220</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
       <c r="A42" s="1">
         <v>5201</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D42" s="1">
         <v>1220</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
       <c r="A43" s="1">
         <v>5251</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D43" s="1">
         <v>1220</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
       <c r="A44" s="1">
         <v>5381</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D44" s="1">
         <v>1220</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
       <c r="A45" s="1">
         <v>5391</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D45" s="1">
         <v>1220</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
       <c r="A46" s="1">
         <v>5401</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D46" s="1">
         <v>1220</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
       <c r="A47" s="1">
         <v>5511</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D47" s="1">
         <v>1220</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
       <c r="A48" s="1">
         <v>1481</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D48" s="1">
         <v>1480</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
       <c r="A49" s="1">
         <v>2281</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D49" s="1">
         <v>1480</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
       <c r="A50" s="1">
         <v>2421</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D50" s="1">
         <v>1480</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
       <c r="A51" s="1">
         <v>4091</v>
       </c>
       <c r="B51" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C51" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="D51" s="1">
         <v>1480</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
       <c r="A52" s="1">
         <v>4101</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D52" s="1">
         <v>1480</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
       <c r="A53" s="1">
         <v>4251</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D53" s="1">
         <v>1480</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
       <c r="A54" s="1">
         <v>4421</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D54" s="1">
         <v>1480</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
       <c r="A55" s="1">
         <v>4601</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D55" s="1">
         <v>1480</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
       <c r="A56" s="1">
         <v>4701</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D56" s="1">
         <v>1480</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
       <c r="A57" s="1">
         <v>1261</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D57" s="1">
         <v>1260</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
       <c r="A58" s="1">
         <v>2151</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D58" s="1">
         <v>1260</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
       <c r="A59" s="1">
         <v>2161</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D59" s="1">
         <v>1260</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
       <c r="A60" s="1">
         <v>2311</v>
       </c>
       <c r="B60" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C60" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>68</v>
       </c>
       <c r="D60" s="1">
         <v>1260</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
       <c r="A61" s="1">
         <v>2351</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D61" s="1">
         <v>1260</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
       <c r="A62" s="1">
         <v>1541</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D62" s="1">
         <v>1540</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
       <c r="A63" s="1">
         <v>1191</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D63" s="1">
         <v>1190</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
       <c r="A64" s="1">
         <v>1911</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D64" s="1">
         <v>1190</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
       <c r="A65" s="1">
         <v>1915</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D65" s="1">
         <v>1190</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
       <c r="A66" s="1">
         <v>1916</v>
       </c>
       <c r="B66" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C66" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>76</v>
       </c>
       <c r="D66" s="1">
         <v>1190</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
       <c r="A67" s="2">
         <v>1917</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D67" s="2">
         <v>1190</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
       <c r="A68" s="1">
         <v>4621</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D68" s="1">
         <v>1190</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
       <c r="A69" s="1">
         <v>4651</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D69" s="1">
         <v>1190</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
       <c r="A70" s="1">
         <v>4721</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D70" s="1">
         <v>1190</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
       <c r="A71" s="1">
         <v>1071</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D71" s="1">
         <v>1070</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
       <c r="A72" s="1">
         <v>1631</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D72" s="1">
         <v>1630</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
       <c r="A73" s="1">
         <v>1491</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D73" s="1">
         <v>1490</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
       <c r="A74" s="1">
         <v>1301</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>129</v>
+        <v>94</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="D74" s="1">
         <v>1300</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
       <c r="A75" s="2">
         <v>2301</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>150</v>
+        <v>96</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="D75" s="2">
         <v>1300</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
       <c r="A76" s="1">
         <v>2431</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>131</v>
+        <v>97</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="D76" s="1">
         <v>1300</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
       <c r="A77" s="1">
         <v>2461</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>132</v>
+        <v>98</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="D77" s="1">
         <v>1300</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5">
       <c r="A78" s="1">
         <v>4331</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>133</v>
+        <v>99</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="D78" s="1">
         <v>1300</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5">
       <c r="A79" s="1">
         <v>4381</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>134</v>
+        <v>100</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="D79" s="1">
         <v>1300</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5">
       <c r="A80" s="1">
         <v>4631</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>135</v>
+        <v>101</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="D80" s="1">
         <v>1300</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5">
       <c r="A81" s="1">
         <v>4641</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>136</v>
+        <v>102</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="D81" s="1">
         <v>1300</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5">
       <c r="A82" s="1">
         <v>5261</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>137</v>
+        <v>103</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="D82" s="1">
         <v>1300</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5">
       <c r="A83" s="1">
         <v>2471</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>148</v>
+        <v>104</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="D83" s="1">
         <v>1300</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5">
       <c r="A84" s="1">
         <v>1451</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="D84" s="1">
         <v>1450</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
       <c r="A85" s="1">
         <v>4141</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="D85" s="1">
         <v>1450</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
       <c r="A86" s="1">
         <v>4321</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="D86" s="1">
         <v>1450</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
       <c r="A87" s="1">
         <v>4691</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="D87" s="1">
         <v>1450</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5">
       <c r="A88" s="1">
         <v>1371</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="D88" s="1">
         <v>1370</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5">
       <c r="A89" s="1">
         <v>2091</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="D89" s="1">
         <v>1370</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5">
       <c r="A90" s="1">
         <v>2101</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="D90" s="1">
         <v>1370</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5">
       <c r="A91" s="1">
         <v>2241</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="D91" s="1">
         <v>1370</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5">
       <c r="A92" s="1">
         <v>2441</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="D92" s="1">
         <v>1370</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5">
       <c r="A93" s="1">
         <v>4341</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="D93" s="1">
         <v>1370</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5">
       <c r="A94" s="1">
         <v>4761</v>
       </c>
       <c r="B94" t="s">
-        <v>152</v>
+        <v>117</v>
       </c>
       <c r="C94" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="D94">
         <v>1370</v>
       </c>
       <c r="E94" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5">
       <c r="A95" s="1">
         <v>1091</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="D95" s="1">
         <v>1090</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5">
       <c r="A96" s="1">
         <v>4441</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="D96" s="1">
         <v>1090</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5">
       <c r="A97" s="1">
         <v>4451</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="D97" s="1">
         <v>1090</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5">
       <c r="A98" s="1">
         <v>4731</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>146</v>
+        <v>123</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="D98" s="1">
         <v>1090</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5">
       <c r="A99" s="1">
         <v>1101</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
       <c r="D99" s="1">
         <v>1100</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5">
       <c r="A100" s="1">
         <v>1501</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="D100" s="1">
         <v>1500</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5">
       <c r="A101" s="1">
         <v>1941</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="D101" s="1">
         <v>1500</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5">
       <c r="A102" s="1">
         <v>2011</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="D102" s="1">
         <v>1500</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5">
       <c r="A103" s="1">
         <v>2061</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="D103" s="1">
         <v>1500</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5">
       <c r="A104" s="1">
         <v>2331</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="D104" s="1">
         <v>1500</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5">
       <c r="A105" s="1">
         <v>4551</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="D105" s="1">
         <v>1500</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5">
       <c r="A106" s="1">
         <v>4711</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="D106" s="1">
         <v>1500</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5">
       <c r="A107" s="1">
         <v>5141</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="D107" s="1">
         <v>1500</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5">
       <c r="A108" s="1">
         <v>2781</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="D108">
         <v>1500</v>
       </c>
       <c r="E108" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5">
       <c r="A109" s="1">
         <v>1511</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="D109" s="1">
         <v>1510</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5">
       <c r="A110" s="1">
         <v>1251</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="D110" s="1">
         <v>1250</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5">
       <c r="A111" s="1">
         <v>2121</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="D111" s="1">
         <v>1250</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5">
       <c r="A112" s="1">
         <v>4541</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="D112" s="1">
         <v>1250</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5">
       <c r="A113" s="1">
         <v>1991</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="D113" s="1">
         <v>1990</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5">
       <c r="A114" s="1">
         <v>2261</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>123</v>
+        <v>141</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="D114" s="1">
         <v>1320</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5">
       <c r="A115" s="1">
         <v>2271</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>126</v>
+        <v>144</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="D115" s="1">
         <v>1320</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5">
       <c r="A116" s="1">
         <v>2321</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="D116" s="1">
         <v>1320</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5">
       <c r="A117" s="1">
         <v>4291</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="D117" s="1">
         <v>1320</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5">
       <c r="A118" s="1">
         <v>1021</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="D118" s="1">
         <v>1020</v>
       </c>
       <c r="E118" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5">
       <c r="A119" s="1">
         <v>4611</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="D119" s="1">
         <v>1020</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5">
       <c r="A120" s="1">
         <v>1031</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="D120" s="1">
         <v>1030</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5">
       <c r="A121" s="1">
         <v>4031</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="D121" s="1">
         <v>1030</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5">
       <c r="A122" s="1">
         <v>1051</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="D122" s="1">
         <v>1050</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -3016,6 +3017,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B08D58FADB61F04EBBB4F355C06EFBED" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="b1e0f6055e0e9a4b9e75d6c71ee7de91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6f4338ef-addb-4c87-aefe-1895241b335f" xmlns:ns3="b91e7f20-fe0a-487d-91a9-605ac1c64acf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b43930f3490e4d4da1ab3f8da7df6f51" ns2:_="" ns3:_="">
     <xsd:import namespace="6f4338ef-addb-4c87-aefe-1895241b335f"/>
@@ -3276,66 +3297,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32A8BD50-45B3-45F1-BF54-8EA14AE06CFE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
-    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C50C5F39-ECEB-47DE-9610-74B8B293C0D0}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C50C5F39-ECEB-47DE-9610-74B8B293C0D0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC85FD73-D9CF-450C-8F57-71B83A4AFF06}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC85FD73-D9CF-450C-8F57-71B83A4AFF06}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32A8BD50-45B3-45F1-BF54-8EA14AE06CFE}"/>
 </file>
</xml_diff>

<commit_message>
Update data package at: 2026-09-25T19:32:13Z
</commit_message>
<xml_diff>
--- a/data-raw/desc_Setor_UO_Orgao.xlsx
+++ b/data-raw/desc_Setor_UO_Orgao.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\x1569275\CAMG\Splor Geral - @dcppn\00- DCPPN 2027\PPAG e LOA 2027\Dados para Volumes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cecad365.sharepoint.com/sites/Splor/Documentos Compartilhados/General/@dcppn/00- DCPPN 2027/PPAG e LOA 2027/Dados para Volumes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_67BEBA03C2A83042867FE281EC8FE06AF5979440" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_67BEBA03C2A83042867FE281EC8FE06AF5979440" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64F9F1C0-2361-4B69-9929-A26E6E44376B}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Setor_UO_Órgão" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Setor_UO_Órgão!$A$1:$E$122</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Setor_UO_Órgão!$A$1:$E$123</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -510,7 +510,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -611,7 +611,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabela2" displayName="Tabela2" ref="A1:E122" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabela2" displayName="Tabela2" ref="A1:E123" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E122">
     <sortCondition ref="C1:C122"/>
   </sortState>
@@ -627,9 +627,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -667,7 +667,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -773,7 +773,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -915,7 +915,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -924,16 +924,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E122"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="63" style="1" customWidth="1"/>
-    <col min="3" max="3" width="46.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="73.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="46.88671875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="73.44140625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -950,7 +950,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1081</v>
       </c>
@@ -967,7 +967,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>4751</v>
       </c>
@@ -984,7 +984,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>1231</v>
       </c>
@@ -1001,7 +1001,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>2371</v>
       </c>
@@ -1018,7 +1018,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>3041</v>
       </c>
@@ -1035,7 +1035,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>3051</v>
       </c>
@@ -1052,7 +1052,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>4171</v>
       </c>
@@ -1069,7 +1069,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>1011</v>
       </c>
@@ -1086,7 +1086,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>2361</v>
       </c>
@@ -1103,7 +1103,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>4121</v>
       </c>
@@ -1120,7 +1120,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>1721</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>1951</v>
       </c>
@@ -1154,7 +1154,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>1711</v>
       </c>
@@ -1171,7 +1171,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>2211</v>
       </c>
@@ -1188,7 +1188,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>3151</v>
       </c>
@@ -1205,7 +1205,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>1521</v>
       </c>
@@ -1222,7 +1222,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>1401</v>
       </c>
@@ -1239,7 +1239,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>1271</v>
       </c>
@@ -1256,7 +1256,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>2171</v>
       </c>
@@ -1273,7 +1273,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>2181</v>
       </c>
@@ -1290,7 +1290,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>2201</v>
       </c>
@@ -1307,7 +1307,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>4151</v>
       </c>
@@ -1324,7 +1324,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>4491</v>
       </c>
@@ -1341,7 +1341,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>1441</v>
       </c>
@@ -1358,7 +1358,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>4741</v>
       </c>
@@ -1375,7 +1375,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>1221</v>
       </c>
@@ -1392,7 +1392,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>2041</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>2071</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>2251</v>
       </c>
@@ -1443,7 +1443,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>4111</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>4531</v>
       </c>
@@ -1477,7 +1477,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>4661</v>
       </c>
@@ -1494,7 +1494,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>4671</v>
       </c>
@@ -1511,7 +1511,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>5011</v>
       </c>
@@ -1528,7 +1528,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>5031</v>
       </c>
@@ -1545,7 +1545,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>5071</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>5081</v>
       </c>
@@ -1579,7 +1579,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>5121</v>
       </c>
@@ -1596,7 +1596,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>5131</v>
       </c>
@@ -1613,7 +1613,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>5191</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>5201</v>
       </c>
@@ -1647,7 +1647,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>5251</v>
       </c>
@@ -1664,7 +1664,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
         <v>5381</v>
       </c>
@@ -1681,7 +1681,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>5391</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
         <v>5401</v>
       </c>
@@ -1715,7 +1715,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>5511</v>
       </c>
@@ -1732,7 +1732,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
         <v>1481</v>
       </c>
@@ -1749,7 +1749,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
         <v>2281</v>
       </c>
@@ -1766,7 +1766,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
         <v>2421</v>
       </c>
@@ -1783,7 +1783,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
         <v>4091</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
         <v>4101</v>
       </c>
@@ -1817,7 +1817,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
         <v>4251</v>
       </c>
@@ -1834,7 +1834,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
         <v>4421</v>
       </c>
@@ -1851,7 +1851,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
         <v>4601</v>
       </c>
@@ -1868,7 +1868,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
         <v>4701</v>
       </c>
@@ -1885,7 +1885,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
         <v>1261</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="1">
         <v>2151</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="1">
         <v>2161</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="1">
         <v>2311</v>
       </c>
@@ -1953,7 +1953,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="1">
         <v>2351</v>
       </c>
@@ -1970,7 +1970,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="1">
         <v>1541</v>
       </c>
@@ -1987,7 +1987,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="1">
         <v>1191</v>
       </c>
@@ -2004,7 +2004,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="1">
         <v>1911</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="1">
         <v>1915</v>
       </c>
@@ -2038,7 +2038,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="66" spans="1:5">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="1">
         <v>1916</v>
       </c>
@@ -2055,7 +2055,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
         <v>1917</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="68" spans="1:5">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="1">
         <v>4621</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="1">
         <v>4651</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="1">
         <v>4721</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="71" spans="1:5">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="1">
         <v>1071</v>
       </c>
@@ -2140,7 +2140,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="72" spans="1:5">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="1">
         <v>1631</v>
       </c>
@@ -2157,7 +2157,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="73" spans="1:5">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="1">
         <v>1491</v>
       </c>
@@ -2174,7 +2174,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="74" spans="1:5">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="1">
         <v>1301</v>
       </c>
@@ -2191,7 +2191,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="75" spans="1:5">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="2">
         <v>2301</v>
       </c>
@@ -2208,7 +2208,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="76" spans="1:5">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="1">
         <v>2431</v>
       </c>
@@ -2225,7 +2225,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="77" spans="1:5">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" s="1">
         <v>2461</v>
       </c>
@@ -2242,7 +2242,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="78" spans="1:5">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="1">
         <v>4331</v>
       </c>
@@ -2259,7 +2259,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="79" spans="1:5">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="1">
         <v>4381</v>
       </c>
@@ -2276,7 +2276,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="80" spans="1:5">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" s="1">
         <v>4631</v>
       </c>
@@ -2293,7 +2293,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="81" spans="1:5">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="1">
         <v>4641</v>
       </c>
@@ -2310,7 +2310,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="82" spans="1:5">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="1">
         <v>5261</v>
       </c>
@@ -2327,7 +2327,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="83" spans="1:5">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="1">
         <v>2471</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="84" spans="1:5">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="1">
         <v>1451</v>
       </c>
@@ -2361,7 +2361,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="85" spans="1:5">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="1">
         <v>4141</v>
       </c>
@@ -2378,7 +2378,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="86" spans="1:5">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="1">
         <v>4321</v>
       </c>
@@ -2395,7 +2395,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="87" spans="1:5">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="1">
         <v>4691</v>
       </c>
@@ -2412,7 +2412,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="88" spans="1:5">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" s="1">
         <v>1371</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="89" spans="1:5">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" s="1">
         <v>2091</v>
       </c>
@@ -2446,7 +2446,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="90" spans="1:5">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="1">
         <v>2101</v>
       </c>
@@ -2463,7 +2463,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="91" spans="1:5">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" s="1">
         <v>2241</v>
       </c>
@@ -2480,7 +2480,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="92" spans="1:5">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" s="1">
         <v>2441</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="93" spans="1:5">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" s="1">
         <v>4341</v>
       </c>
@@ -2514,7 +2514,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="94" spans="1:5">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="1">
         <v>4761</v>
       </c>
@@ -2531,7 +2531,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="95" spans="1:5">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" s="1">
         <v>1091</v>
       </c>
@@ -2548,7 +2548,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="96" spans="1:5">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="1">
         <v>4441</v>
       </c>
@@ -2565,7 +2565,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="97" spans="1:5">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" s="1">
         <v>4451</v>
       </c>
@@ -2582,7 +2582,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="98" spans="1:5">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" s="1">
         <v>4731</v>
       </c>
@@ -2599,7 +2599,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="99" spans="1:5">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" s="1">
         <v>1101</v>
       </c>
@@ -2616,7 +2616,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="100" spans="1:5">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" s="1">
         <v>1501</v>
       </c>
@@ -2633,7 +2633,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="101" spans="1:5">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101" s="1">
         <v>1941</v>
       </c>
@@ -2650,7 +2650,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="102" spans="1:5">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102" s="1">
         <v>2011</v>
       </c>
@@ -2667,7 +2667,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="103" spans="1:5">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A103" s="1">
         <v>2061</v>
       </c>
@@ -2684,7 +2684,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="104" spans="1:5">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A104" s="1">
         <v>2331</v>
       </c>
@@ -2701,7 +2701,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="105" spans="1:5">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A105" s="1">
         <v>4551</v>
       </c>
@@ -2718,7 +2718,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="106" spans="1:5">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A106" s="1">
         <v>4711</v>
       </c>
@@ -2735,7 +2735,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="107" spans="1:5">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107" s="1">
         <v>5141</v>
       </c>
@@ -2752,9 +2752,9 @@
         <v>126</v>
       </c>
     </row>
-    <row r="108" spans="1:5">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A108" s="1">
-        <v>2781</v>
+        <v>2481</v>
       </c>
       <c r="B108" s="1" t="s">
         <v>135</v>
@@ -2769,7 +2769,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="109" spans="1:5">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A109" s="1">
         <v>1511</v>
       </c>
@@ -2786,7 +2786,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="110" spans="1:5">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110" s="1">
         <v>1251</v>
       </c>
@@ -2803,7 +2803,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="111" spans="1:5">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A111" s="1">
         <v>2121</v>
       </c>
@@ -2820,7 +2820,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="112" spans="1:5">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112" s="1">
         <v>4541</v>
       </c>
@@ -2837,7 +2837,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="113" spans="1:5">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A113" s="1">
         <v>1991</v>
       </c>
@@ -2854,7 +2854,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="114" spans="1:5">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A114" s="1">
         <v>2261</v>
       </c>
@@ -2871,7 +2871,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="115" spans="1:5">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A115" s="1">
         <v>2271</v>
       </c>
@@ -2888,7 +2888,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="116" spans="1:5">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A116" s="1">
         <v>2321</v>
       </c>
@@ -2905,7 +2905,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="117" spans="1:5">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A117" s="1">
         <v>4291</v>
       </c>
@@ -2922,7 +2922,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="118" spans="1:5">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A118" s="1">
         <v>1021</v>
       </c>
@@ -2939,7 +2939,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="119" spans="1:5">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A119" s="1">
         <v>4611</v>
       </c>
@@ -2956,7 +2956,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="120" spans="1:5">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A120" s="1">
         <v>1031</v>
       </c>
@@ -2973,7 +2973,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="121" spans="1:5">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A121" s="1">
         <v>4031</v>
       </c>
@@ -2990,7 +2990,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="122" spans="1:5">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A122" s="1">
         <v>1051</v>
       </c>
@@ -3017,15 +3017,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
@@ -3034,6 +3025,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3298,13 +3298,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C50C5F39-ECEB-47DE-9610-74B8B293C0D0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC85FD73-D9CF-450C-8F57-71B83A4AFF06}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC85FD73-D9CF-450C-8F57-71B83A4AFF06}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C50C5F39-ECEB-47DE-9610-74B8B293C0D0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32A8BD50-45B3-45F1-BF54-8EA14AE06CFE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32A8BD50-45B3-45F1-BF54-8EA14AE06CFE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>